<commit_message>
fix: correct product categories and add auto-filter to pricing analysis
- Fixed Cetaphil creams, Aveeno Lotion, Crest Toothpaste, Revlon Hair Color
  wrongly placed under BODY WASH — now correctly in BODY LOTION, PERSONAL CARE, HAIR
- Added CATEGORY_OVERRIDES map for products missing from spreadsheet category list
- Spreadsheet category is now primary source, file-parsed is fallback only
- Added AutoFilter dropdowns to all columns for easy sorting/filtering in Excel
- Regenerated AmericanSelect_PricingAnalysis_June2026.xlsx with all fixes applied

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AmericanSelect_PricingAnalysis_June2026.xlsx
+++ b/AmericanSelect_PricingAnalysis_June2026.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C2DD528-09E5-4CC3-9CE0-F0FDC10665F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4051E3DA-1DA6-4F8A-9945-3BE872968B3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="23520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1790,7 +1790,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>29</v>
       </c>
@@ -3056,7 +3056,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="52" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="10" t="s">
         <v>91</v>
       </c>
@@ -3082,7 +3082,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
         <v>91</v>
       </c>
@@ -3108,7 +3108,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
         <v>91</v>
       </c>
@@ -3134,7 +3134,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="55" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
         <v>91</v>
       </c>
@@ -3160,7 +3160,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="56" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="10" t="s">
         <v>91</v>
       </c>
@@ -3186,7 +3186,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="57" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="14" t="s">
         <v>91</v>
       </c>
@@ -3212,7 +3212,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="58" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="10" t="s">
         <v>91</v>
       </c>
@@ -3390,7 +3390,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="65" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="14" t="s">
         <v>91</v>
       </c>
@@ -3416,7 +3416,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="66" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="10" t="s">
         <v>91</v>
       </c>
@@ -3442,7 +3442,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="14" t="s">
         <v>91</v>
       </c>
@@ -3702,7 +3702,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="77" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="14" t="s">
         <v>123</v>
       </c>
@@ -3728,7 +3728,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="78" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="10" t="s">
         <v>123</v>
       </c>
@@ -3754,7 +3754,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="79" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="14" t="s">
         <v>123</v>
       </c>
@@ -4040,7 +4040,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="90" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="10" t="s">
         <v>144</v>
       </c>
@@ -4066,7 +4066,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="91" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="14" t="s">
         <v>144</v>
       </c>
@@ -4092,7 +4092,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="92" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="10" t="s">
         <v>144</v>
       </c>
@@ -4140,7 +4140,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="94" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="10" t="s">
         <v>144</v>
       </c>
@@ -4210,7 +4210,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="97" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="14" t="s">
         <v>144</v>
       </c>
@@ -4258,7 +4258,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="99" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="14" t="s">
         <v>144</v>
       </c>
@@ -4284,7 +4284,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="100" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="10" t="s">
         <v>144</v>
       </c>
@@ -4310,7 +4310,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="101" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="14" t="s">
         <v>144</v>
       </c>
@@ -4358,7 +4358,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="103" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="14" t="s">
         <v>144</v>
       </c>
@@ -4384,7 +4384,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="104" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="10" t="s">
         <v>144</v>
       </c>
@@ -4410,7 +4410,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="105" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="14" t="s">
         <v>144</v>
       </c>
@@ -4458,7 +4458,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="107" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="14" t="s">
         <v>144</v>
       </c>
@@ -4484,7 +4484,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="108" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="10" t="s">
         <v>144</v>
       </c>
@@ -4510,7 +4510,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="109" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="14" t="s">
         <v>144</v>
       </c>
@@ -4580,7 +4580,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="112" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="10" t="s">
         <v>144</v>
       </c>
@@ -4672,7 +4672,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="116" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="10" t="s">
         <v>144</v>
       </c>
@@ -4698,7 +4698,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="117" spans="1:8" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="14" t="s">
         <v>144</v>
       </c>
@@ -4724,7 +4724,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="118" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="10" t="s">
         <v>144</v>
       </c>
@@ -4750,7 +4750,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="119" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="14" t="s">
         <v>144</v>
       </c>
@@ -4776,7 +4776,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="120" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="10" t="s">
         <v>144</v>
       </c>
@@ -5076,7 +5076,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="132" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="10" t="s">
         <v>204</v>
       </c>
@@ -5102,7 +5102,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="133" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="14" t="s">
         <v>204</v>
       </c>
@@ -5128,7 +5128,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="134" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" s="10" t="s">
         <v>204</v>
       </c>
@@ -5202,7 +5202,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="137" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="14" t="s">
         <v>211</v>
       </c>
@@ -5228,7 +5228,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="138" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="10" t="s">
         <v>211</v>
       </c>
@@ -5254,7 +5254,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="139" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="14" t="s">
         <v>211</v>
       </c>
@@ -5280,7 +5280,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="140" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="10" t="s">
         <v>211</v>
       </c>
@@ -5328,7 +5328,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="142" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142" s="10" t="s">
         <v>211</v>
       </c>
@@ -5398,7 +5398,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="145" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A145" s="14" t="s">
         <v>222</v>
       </c>
@@ -5424,7 +5424,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="146" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="10" t="s">
         <v>222</v>
       </c>
@@ -5550,7 +5550,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="151" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A151" s="14" t="s">
         <v>229</v>
       </c>
@@ -5620,7 +5620,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="154" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A154" s="10" t="s">
         <v>229</v>
       </c>
@@ -5738,7 +5738,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="159" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A159" s="14" t="s">
         <v>229</v>
       </c>
@@ -5786,7 +5786,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="161" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A161" s="14" t="s">
         <v>229</v>
       </c>
@@ -5860,7 +5860,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="164" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A164" s="10" t="s">
         <v>244</v>
       </c>
@@ -5886,7 +5886,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="165" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A165" s="14" t="s">
         <v>244</v>
       </c>
@@ -5912,7 +5912,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="166" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A166" s="10" t="s">
         <v>244</v>
       </c>
@@ -5964,7 +5964,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="168" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A168" s="10" t="s">
         <v>244</v>
       </c>
@@ -6016,7 +6016,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="170" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A170" s="10" t="s">
         <v>244</v>
       </c>
@@ -6068,7 +6068,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="172" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A172" s="10" t="s">
         <v>244</v>
       </c>
@@ -6146,7 +6146,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="175" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A175" s="14" t="s">
         <v>244</v>
       </c>
@@ -6172,7 +6172,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="176" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A176" s="10" t="s">
         <v>244</v>
       </c>
@@ -6198,7 +6198,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="177" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A177" s="14" t="s">
         <v>244</v>
       </c>
@@ -6224,7 +6224,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="178" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A178" s="10" t="s">
         <v>244</v>
       </c>
@@ -6276,7 +6276,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="180" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A180" s="10" t="s">
         <v>244</v>
       </c>
@@ -6380,7 +6380,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="184" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A184" s="10" t="s">
         <v>244</v>
       </c>
@@ -6432,7 +6432,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="186" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A186" s="10" t="s">
         <v>244</v>
       </c>
@@ -6458,7 +6458,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="187" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A187" s="14" t="s">
         <v>244</v>
       </c>
@@ -6536,7 +6536,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="190" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A190" s="10" t="s">
         <v>277</v>
       </c>
@@ -6744,7 +6744,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="198" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A198" s="10" t="s">
         <v>277</v>
       </c>
@@ -6796,7 +6796,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="200" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A200" s="10" t="s">
         <v>277</v>
       </c>
@@ -7004,7 +7004,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="208" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A208" s="10" t="s">
         <v>299</v>
       </c>
@@ -7104,7 +7104,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="212" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:8" ht="20.100000000000001" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A212" s="10" t="s">
         <v>299</v>
       </c>
@@ -7160,8 +7160,7 @@
   <autoFilter ref="A1:H213" xr:uid="{00000000-0009-0000-0000-000001000000}">
     <filterColumn colId="7">
       <filters>
-        <filter val="Could go higher"/>
-        <filter val="Slight raise needed"/>
+        <filter val="SELLING AT A LOSS"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>